<commit_message>
feat: add test automation framework v1.0 with core utilities, test cases, and CI workflows
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/Builder/NEMO-24401/NEMO-24401_builder_clone_component_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/Builder/NEMO-24401/NEMO-24401_builder_clone_component_test_cases.xlsx
@@ -357,7 +357,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Code my_comp_01 does not already exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Locate cqaclone1_15junepe1
 4. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
@@ -383,7 +383,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Code comp_2024 does not exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Locate cqaclone1_15junepe1
 4. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
@@ -406,7 +406,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Code comp_a_2_b does not exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Locate cqaclone1_15junepe1
 4. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
@@ -432,7 +432,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Code unique_new_01 does not exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter duplicate: cqaclone1_15junepe1
@@ -456,7 +456,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Ingested cqathorjune10pe1 exists. Code reg_comp_new_01 does not exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter: cqathorjune10pe1 (ingested code)
@@ -480,7 +480,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Code reuse_comp_del_01 does not exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter: reuse_comp_del_01
@@ -505,7 +505,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Code reuse_after_del_comp does not exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Clone cqaclone1_15junepe1 with code: reuse_after_del_comp
 4. Confirm clone success
@@ -530,7 +530,7 @@
     <t>Logged in as Admin. Non-ingested eBook cqacloneebook15june26 and Component cqaclone1_15junepe1 exist. Code reuse_ebook_on_comp_01 does not exist.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to eBooks listing
 3. Clone cqacloneebook15june26 with code: reuse_ebook_on_comp_01
 4. Confirm eBook clone success
@@ -556,7 +556,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter whitespace only (3+ spaces) in Unique Code field
@@ -575,7 +575,7 @@
     <t>Verify the duplicate code error is displayed inline near the code field, not as a browser alert dialog</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter: cqaclone1_15junepe1 (own code)
@@ -595,7 +595,7 @@
     <t>Verify an inline uniqueness error is shown when cloning using the source component's own existing code</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter code: cqaclone1_15junepe1
@@ -617,7 +617,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Umbrella cqaumbrellaforautotest15june2026 exists.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter code: cqaumbrellaforautotest15june2026
@@ -639,7 +639,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Non-ingested eBook cqacloneebook15june26 exists.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter code: cqacloneebook15june26
@@ -655,7 +655,7 @@
     <t>Verify a required-field error is shown when the unique code field is left empty</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Leave Unique Code field empty
@@ -671,7 +671,7 @@
     <t>Verify a format error is shown when the unique code contains uppercase letters</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter code: MyComp_Invalid
@@ -687,7 +687,7 @@
     <t>Verify a format error is shown when the unique code contains special characters</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter code: comp-one@test
@@ -706,7 +706,7 @@
     <t>Logged in as Admin on Builder Thor. Ingested component cqathorjune10pe1 visible in listing.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Locate ingested component cqathorjune10pe1
 4. Open action menu [ASSUMED]
@@ -728,7 +728,7 @@
     <t>Logged in as Admin (harishthoradmin) on Builder Thor. Component "cqaclone1_15junepe1" (non-ingested) visible in listing. Ingested cqathorjune10pe1 exists.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Navigate to Components listing page [ASSUMED: left nav or top menu]
 3. Click Clone action for cqaclone1_15junepe1 [ASSUMED: context menu / action button]
 4. Enter code: cqathorjune10pe1
@@ -777,7 +777,7 @@
     <t>Logged in as Admin on Builder Thor. Component cqaclone1_15junepe1 (non-ingested) visible. Code family_comp_01 does not already exist anywhere.</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Left pane: click Families [ASSUMED]
 3. Click Create a Family [ASSUMED]
 4. Enter unique code: family_comp_01 (lowercase letters + numbers)
@@ -803,7 +803,7 @@
     <t>Logged in as Admin on Builder Thor. Component cqaclone1_15junepe1 visible. Family with code family_comp_01 exists (created in TST_NEMO24401_TC_19 or fresh).</t>
   </si>
   <si>
-    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / C0&gt;pr0!899
+    <t>1. Login: https://asgard-thor-builder.comprodls.com/2024/pre-login | Org: Cambridge One | Confirm | IdP: harishthoradmin / {{env.BLDR_THOR_VALIDADMIN_PASSWORD}}
 2. Left pane: click Families [ASSUMED]
 3. Locate Family family_comp_01
 4. Click Delete action for Family family_comp_01 [ASSUMED]

</xml_diff>